<commit_message>
Add five-agent BFM workflow and Gmail integration
</commit_message>
<xml_diff>
--- a/data/bfm_demo_data.xlsx
+++ b/data/bfm_demo_data.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Accounts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Revenue Realization" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Billing Tracker" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Collection Tracker" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Projects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Billing Milestones" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Collections" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Thresholds" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,43 +441,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Master account directory with targets and ownership</t>
+          <t>Account owners, delivery units, client contacts, and monthly targets</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Revenue Realization</t>
+          <t>Projects</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Project-level revenue monitoring inputs</t>
+          <t>Raw revenue, trend, forecast, and billing ownership inputs</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Billing Tracker</t>
+          <t>Billing Milestones</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Milestone billing and unbilled revenue tracking</t>
+          <t>Milestone completion and billing trigger records</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Collection Tracker</t>
+          <t>Collections</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Invoice collections and overdue monitoring</t>
+          <t>Invoice and collection tracking records</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Thresholds</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Agent-specific dynamic risk thresholds editable from the UI</t>
         </is>
       </c>
     </row>
@@ -491,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,10 +535,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Client Contact Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Client Contact Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Account Monthly Target</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Contract Value</t>
         </is>
@@ -534,232 +557,259 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>PepsiCo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Life Sciences</t>
+          <t>Consumer Goods</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Enterprise Platforms</t>
+          <t>Data &amp; AI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kavya Nair</t>
+          <t>Priya Sharma</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>kavya.nair@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>280000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>4500000</v>
+          <t>priya.sharma@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Daniel Cooper</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>daniel.cooper@pepsico-demo.local</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="I2" t="n">
+        <v>6000000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Comcast</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Networking</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cyber Defense</t>
+          <t>Digital Engineering</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sanjay Patel</t>
+          <t>Neha Iyer</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sanjay.patel@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>290000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>3950000</v>
+          <t>neha.iyer@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Melissa Grant</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>melissa.grant@comcast-demo.local</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1650000</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5100000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Comcast</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Banking</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Digital Engineering</t>
+          <t>Managed Services</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Neha Iyer</t>
+          <t>Rohit Desai</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>neha.iyer@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>310000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>4100000</v>
+          <t>rohit.desai@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Liam Porter</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>liam.porter@hsbc-demo.local</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4750000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Banking</t>
+          <t>Life Sciences</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Managed Services</t>
+          <t>Enterprise Platforms</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Rohit Desai</t>
+          <t>Kavya Nair</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>rohit.desai@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>340000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4700000</v>
+          <t>kavya.nair@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sophia Reed</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>sophia.reed@astrazeneca-demo.local</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5500000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Johnson Controls</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industrial Technology</t>
+          <t>Networking</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cloud Ops</t>
+          <t>Cyber Defense</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Arjun Mehta</t>
+          <t>Sanjay Patel</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>arjun.mehta@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>260000</v>
-      </c>
-      <c r="G6" t="n">
-        <v>3500000</v>
+          <t>sanjay.patel@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Victor Hill</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>victor.hill@cisco-demo.local</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4550000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PepsiCo</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Consumer Goods</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Data &amp; AI</t>
+          <t>Commerce Platforms</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>Ananya Rao</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>priya.sharma@bfmdemo.local</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>420000</v>
-      </c>
-      <c r="G7" t="n">
-        <v>5100000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Retail</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Commerce Platforms</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Ananya Rao</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
           <t>ananya.rao@bfmdemo.local</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>280000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>3800000</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Grace Miller</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>grace.miller@target-demo.local</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>780000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2300000</v>
       </c>
     </row>
   </sheetData>
@@ -773,7 +823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -799,65 +849,75 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Billing Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Billing Owner</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Billing Owner Email</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Contract Value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Revenue Plan (Month)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Revenue Plan (Quarter)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Revenue Recognized</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Revenue Remaining</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Revenue Forecast</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Revenue Gap</t>
-        </is>
-      </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Revenue Completion %</t>
+          <t>Recognized Last 7 Days</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Revenue Burn Rate</t>
+          <t>Recognized Last 30 Days</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Pending Pipeline</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Forecast Bias</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>Last Revenue Update</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Billing Cycle Days</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
@@ -871,62 +931,74 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PEP-AI-101</t>
+          <t>PRJ-4456</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Demand Forecasting Modernization</t>
+          <t>Global Data Platform Rollout</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI Platforms</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>2700000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>220000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>660000</v>
+          <t>Data Modernization</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aditya Bose</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>aditya.bose@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H2" t="n">
-        <v>173000</v>
+        <v>3600000</v>
       </c>
       <c r="I2" t="n">
-        <v>47000</v>
+        <v>1400000</v>
       </c>
       <c r="J2" t="n">
-        <v>189000</v>
+        <v>4200000</v>
       </c>
       <c r="K2" t="n">
-        <v>-31000</v>
+        <v>1100000</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7864</v>
+        <v>35000</v>
       </c>
       <c r="M2" t="n">
-        <v>43250</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
+        <v>140000</v>
+      </c>
+      <c r="N2" t="n">
+        <v>30000</v>
       </c>
       <c r="O2" t="n">
-        <v>30</v>
+        <v>0.95</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>2027-03-11</t>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>7</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2027-05-11</t>
         </is>
       </c>
     </row>
@@ -938,464 +1010,548 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PEP-DA-204</t>
+          <t>PRJ-4521</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Retail Data Hub Rollout</t>
+          <t>Retail Insights Factory</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Data Engineering</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+          <t>Analytics Engineering</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Time &amp; Material</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Meera Jain</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>meera.jain@bfmdemo.local</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
         <v>2400000</v>
       </c>
-      <c r="F3" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>600000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>153000</v>
-      </c>
       <c r="I3" t="n">
-        <v>47000</v>
+        <v>1000000</v>
       </c>
       <c r="J3" t="n">
-        <v>172000</v>
+        <v>3000000</v>
       </c>
       <c r="K3" t="n">
-        <v>-28000</v>
+        <v>800000</v>
       </c>
       <c r="L3" t="n">
-        <v>0.765</v>
+        <v>25000</v>
       </c>
       <c r="M3" t="n">
-        <v>38250</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
+        <v>108000</v>
+      </c>
+      <c r="N3" t="n">
+        <v>10000</v>
       </c>
       <c r="O3" t="n">
-        <v>45</v>
+        <v>0.88</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2025-06-29</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2027-07-09</t>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>14</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2027-03-12</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Johnson Controls</t>
+          <t>Comcast</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>JCI-OPS-310</t>
+          <t>PRJ-4588</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Facilities Cloud Operations</t>
+          <t>Customer App Modernization</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Managed Services</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>1900000</v>
-      </c>
-      <c r="F4" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>450000</v>
+          <t>Digital Product Engineering</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Kiran Sethi</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>kiran.sethi@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>149000</v>
+        <v>2900000</v>
       </c>
       <c r="I4" t="n">
-        <v>1000</v>
+        <v>900000</v>
       </c>
       <c r="J4" t="n">
-        <v>154000</v>
+        <v>2700000</v>
       </c>
       <c r="K4" t="n">
-        <v>4000</v>
+        <v>690000</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9933</v>
+        <v>40000</v>
       </c>
       <c r="M4" t="n">
-        <v>37250</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
+        <v>155000</v>
+      </c>
+      <c r="N4" t="n">
+        <v>80000</v>
       </c>
       <c r="O4" t="n">
-        <v>30</v>
+        <v>1.02</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2025-04-10</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2027-05-10</t>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2025-05-31</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2027-04-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Johnson Controls</t>
+          <t>Comcast</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JCI-CLO-115</t>
+          <t>PRJ-4620</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Workplace IoT Integration</t>
+          <t>Network AIOps Pilot</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Cloud Transformation</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>1600000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>110000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>330000</v>
+          <t>Platform Engineering</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Time &amp; Material</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Rashmi Gupta</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>rashmi.gupta@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>106000</v>
+        <v>2200000</v>
       </c>
       <c r="I5" t="n">
-        <v>4000</v>
+        <v>750000</v>
       </c>
       <c r="J5" t="n">
-        <v>114000</v>
+        <v>2250000</v>
       </c>
       <c r="K5" t="n">
-        <v>4000</v>
+        <v>580000</v>
       </c>
       <c r="L5" t="n">
-        <v>0.9636</v>
+        <v>28000</v>
       </c>
       <c r="M5" t="n">
-        <v>26500</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
+        <v>118000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>45000</v>
       </c>
       <c r="O5" t="n">
-        <v>30</v>
+        <v>0.98</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2025-09-07</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2027-01-10</t>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2027-02-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Comcast</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>COM-DIG-501</t>
+          <t>PRJ-4711</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Customer App Modernization</t>
+          <t>Regulatory Data Platform</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Digital Product Engineering</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>2300000</v>
-      </c>
-      <c r="F6" t="n">
-        <v>170000</v>
-      </c>
-      <c r="G6" t="n">
-        <v>510000</v>
+          <t>Data Platforms</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nikhil Verma</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>nikhil.verma@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H6" t="n">
-        <v>136000</v>
+        <v>2700000</v>
       </c>
       <c r="I6" t="n">
-        <v>34000</v>
+        <v>850000</v>
       </c>
       <c r="J6" t="n">
-        <v>152000</v>
+        <v>2550000</v>
       </c>
       <c r="K6" t="n">
-        <v>-18000</v>
+        <v>780000</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8</v>
+        <v>25000</v>
       </c>
       <c r="M6" t="n">
-        <v>34000</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
+        <v>100000</v>
+      </c>
+      <c r="N6" t="n">
+        <v>35000</v>
       </c>
       <c r="O6" t="n">
-        <v>21</v>
+        <v>1.03</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2027-04-20</t>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2025-05-11</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2027-05-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Comcast</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>COM-AIO-118</t>
+          <t>PRJ-4730</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Network AIOps Pilot</t>
+          <t>Treasury Operations Support</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Platform Engineering</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>1800000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>140000</v>
-      </c>
-      <c r="G7" t="n">
-        <v>420000</v>
+          <t>Finance Ops</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Time &amp; Material</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Asha Menon</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>asha.menon@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>108000</v>
+        <v>2050000</v>
       </c>
       <c r="I7" t="n">
-        <v>32000</v>
+        <v>650000</v>
       </c>
       <c r="J7" t="n">
-        <v>127000</v>
+        <v>1950000</v>
       </c>
       <c r="K7" t="n">
-        <v>-13000</v>
+        <v>590000</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7714</v>
+        <v>18000</v>
       </c>
       <c r="M7" t="n">
-        <v>27000</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
+        <v>88000</v>
+      </c>
+      <c r="N7" t="n">
+        <v>20000</v>
       </c>
       <c r="O7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2027-02-09</t>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>14</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2027-04-11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HSB-DAT-220</t>
+          <t>PRJ-4870</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Regulatory Data Platform</t>
+          <t>SAP Finance Transformation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Data Modernization</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2600000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>180000</v>
-      </c>
-      <c r="G8" t="n">
-        <v>540000</v>
+          <t>ERP Modernization</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ritu Chopra</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ritu.chopra@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H8" t="n">
-        <v>168000</v>
+        <v>3100000</v>
       </c>
       <c r="I8" t="n">
-        <v>12000</v>
+        <v>980000</v>
       </c>
       <c r="J8" t="n">
-        <v>185000</v>
+        <v>2940000</v>
       </c>
       <c r="K8" t="n">
-        <v>5000</v>
+        <v>720000</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9333</v>
+        <v>30000</v>
       </c>
       <c r="M8" t="n">
-        <v>42000</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
+        <v>128000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>55000</v>
       </c>
       <c r="O8" t="n">
-        <v>30</v>
+        <v>0.9</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2025-05-10</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>2027-07-29</t>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2025-04-21</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2027-07-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HSB-FIN-804</t>
+          <t>PRJ-4902</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Treasury Operations Support</t>
+          <t>Clinical Data Lake</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Finance Ops</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>2100000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>160000</v>
-      </c>
-      <c r="G9" t="n">
-        <v>480000</v>
+          <t>Data Platforms</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Time &amp; Material</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Naveen Pillai</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>naveen.pillai@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H9" t="n">
-        <v>138000</v>
+        <v>2400000</v>
       </c>
       <c r="I9" t="n">
-        <v>22000</v>
+        <v>720000</v>
       </c>
       <c r="J9" t="n">
-        <v>151000</v>
+        <v>2160000</v>
       </c>
       <c r="K9" t="n">
-        <v>-9000</v>
+        <v>530000</v>
       </c>
       <c r="L9" t="n">
-        <v>0.8625</v>
+        <v>20000</v>
       </c>
       <c r="M9" t="n">
-        <v>34500</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
+        <v>86000</v>
+      </c>
+      <c r="N9" t="n">
+        <v>60000</v>
       </c>
       <c r="O9" t="n">
-        <v>21</v>
+        <v>0.88</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>2027-05-10</t>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>10</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2027-04-21</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1563,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CSC-CYB-410</t>
+          <t>PRJ-5031</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1420,49 +1576,61 @@
           <t>Cybersecurity</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>145000</v>
-      </c>
-      <c r="G10" t="n">
-        <v>435000</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Harsh Bhatia</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>harsh.bhatia@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H10" t="n">
-        <v>151000</v>
+        <v>2500000</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>830000</v>
       </c>
       <c r="J10" t="n">
-        <v>156000</v>
+        <v>2490000</v>
       </c>
       <c r="K10" t="n">
-        <v>11000</v>
+        <v>810000</v>
       </c>
       <c r="L10" t="n">
-        <v>1.0414</v>
+        <v>18000</v>
       </c>
       <c r="M10" t="n">
-        <v>37750</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-03-15</t>
-        </is>
+        <v>82000</v>
+      </c>
+      <c r="N10" t="n">
+        <v>20000</v>
       </c>
       <c r="O10" t="n">
-        <v>30</v>
+        <v>1.05</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2025-05-20</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>2027-04-10</t>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2027-03-12</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1642,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CSC-NET-870</t>
+          <t>PRJ-5077</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1487,317 +1655,140 @@
           <t>Network Engineering</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>1950000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>145000</v>
-      </c>
-      <c r="G11" t="n">
-        <v>435000</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Time &amp; Material</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Tanya Singh</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>tanya.singh@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H11" t="n">
-        <v>144000</v>
+        <v>2050000</v>
       </c>
       <c r="I11" t="n">
-        <v>1000</v>
+        <v>620000</v>
       </c>
       <c r="J11" t="n">
-        <v>146000</v>
+        <v>1860000</v>
       </c>
       <c r="K11" t="n">
-        <v>1000</v>
+        <v>600000</v>
       </c>
       <c r="L11" t="n">
-        <v>0.9931</v>
+        <v>15000</v>
       </c>
       <c r="M11" t="n">
-        <v>36000</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
+        <v>70000</v>
+      </c>
+      <c r="N11" t="n">
+        <v>10000</v>
       </c>
       <c r="O11" t="n">
-        <v>30</v>
+        <v>1.02</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2027-03-11</t>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>14</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2025-08-09</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2027-02-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AZE-ERP-330</t>
+          <t>PRJ-5105</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SAP Finance Transformation</t>
+          <t>Store Commerce Engine</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ERP Modernization</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>2450000</v>
-      </c>
-      <c r="F12" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G12" t="n">
-        <v>450000</v>
+          <t>Commerce Engineering</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Varun Kapoor</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>varun.kapoor@bfmdemo.local</t>
+        </is>
       </c>
       <c r="H12" t="n">
-        <v>112000</v>
+        <v>2300000</v>
       </c>
       <c r="I12" t="n">
-        <v>38000</v>
+        <v>780000</v>
       </c>
       <c r="J12" t="n">
-        <v>129000</v>
+        <v>2340000</v>
       </c>
       <c r="K12" t="n">
-        <v>-21000</v>
+        <v>745000</v>
       </c>
       <c r="L12" t="n">
-        <v>0.7467</v>
+        <v>20000</v>
       </c>
       <c r="M12" t="n">
-        <v>28000</v>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
+        <v>92000</v>
+      </c>
+      <c r="N12" t="n">
+        <v>15000</v>
       </c>
       <c r="O12" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>2027-08-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AstraZeneca</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>AZE-DAT-731</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Clinical Data Lake</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Data Platforms</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>2050000</v>
-      </c>
-      <c r="F13" t="n">
-        <v>130000</v>
-      </c>
-      <c r="G13" t="n">
-        <v>390000</v>
-      </c>
-      <c r="H13" t="n">
-        <v>106000</v>
-      </c>
-      <c r="I13" t="n">
-        <v>24000</v>
-      </c>
-      <c r="J13" t="n">
-        <v>123000</v>
-      </c>
-      <c r="K13" t="n">
-        <v>-7000</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.8154</v>
-      </c>
-      <c r="M13" t="n">
-        <v>26500</v>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="O13" t="n">
-        <v>21</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>2027-04-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>TGT-COM-610</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Store Commerce Engine</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Commerce Engineering</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>2100000</v>
-      </c>
-      <c r="F14" t="n">
-        <v>160000</v>
-      </c>
-      <c r="G14" t="n">
-        <v>480000</v>
-      </c>
-      <c r="H14" t="n">
-        <v>157000</v>
-      </c>
-      <c r="I14" t="n">
-        <v>3000</v>
-      </c>
-      <c r="J14" t="n">
-        <v>162000</v>
-      </c>
-      <c r="K14" t="n">
-        <v>2000</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.9812</v>
-      </c>
-      <c r="M14" t="n">
-        <v>39250</v>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
-      <c r="O14" t="n">
-        <v>30</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>2025-07-19</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>2027-04-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>TGT-ANA-205</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Retail Analytics Factory</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1700000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>120000</v>
-      </c>
-      <c r="G15" t="n">
-        <v>360000</v>
-      </c>
-      <c r="H15" t="n">
-        <v>113000</v>
-      </c>
-      <c r="I15" t="n">
-        <v>7000</v>
-      </c>
-      <c r="J15" t="n">
-        <v>119000</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.9417</v>
-      </c>
-      <c r="M15" t="n">
-        <v>28250</v>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="O15" t="n">
-        <v>30</v>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>2025-09-17</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>2027-02-19</t>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>7</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>2027-03-12</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1828,547 +1819,602 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Completion Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Billable Amount</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Billed Amount</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Unbilled Amount</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Billing Due Date</t>
+          <t>Invoice Generated</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Billed Date</t>
+          <t>Invoice Number</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Delay Days</t>
+          <t>Invoice Date</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Account Manager Response</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Status Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PEP-AI-101</t>
+          <t>PRJ-4456</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>March data science milestone</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>90000</v>
+          <t>Wave 3 billing package</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>68000</v>
+        <v>220000</v>
       </c>
       <c r="E2" t="n">
-        <v>22000</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>8</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Pending Approval</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Revenue recognized but invoice trigger is pending.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PEP-DA-204</t>
+          <t>PRJ-4456</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wave 2 platform billing</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>78000</v>
+          <t>Data migration sign-off</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>14000</v>
+        <v>200000</v>
       </c>
       <c r="E3" t="n">
-        <v>64000</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>16</v>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Awaiting account manager approval to release invoice.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JCI-OPS-310</t>
+          <t>PRJ-4521</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Monthly cloud operations billing</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>62000</v>
+          <t>Sprint 18 billing lot</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>56000</v>
+        <v>70000</v>
       </c>
       <c r="E4" t="n">
-        <v>6000</v>
+        <v>50000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
+          <t>INV-4521-88</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Ready To Bill</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Partially invoiced while change order is being approved.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JCI-CLO-115</t>
+          <t>PRJ-4588</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Phase gate billing</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>55000</v>
+          <t>Release train 7 sign-off</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>43000</v>
+        <v>180000</v>
       </c>
       <c r="E5" t="n">
-        <v>12000</v>
+        <v>120000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>4</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>INV-4588-17</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Pending Approval</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Residual services effort is pending billing release.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COM-DIG-501</t>
+          <t>PRJ-4620</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sprint 18 billing pack</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>68000</v>
+          <t>Observability milestone</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>31000</v>
+        <v>95000</v>
       </c>
       <c r="E6" t="n">
-        <v>37000</v>
+        <v>40000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>12</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>INV-4620-41</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Pending Client Confirmation</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Invoice created but not fully billed against completed effort.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COM-AIO-118</t>
+          <t>PRJ-4711</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Observability billing batch</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>54000</v>
+          <t>Regulatory release billing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>39000</v>
+        <v>110000</v>
       </c>
       <c r="E7" t="n">
-        <v>15000</v>
+        <v>110000</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>6</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>INV-4711-22</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Delayed</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Billing released on schedule.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HSB-DAT-220</t>
+          <t>PRJ-4730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>March reporting milestone</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>72000</v>
+          <t>Treasury operations monthly pack</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
       </c>
       <c r="D8" t="n">
-        <v>63000</v>
+        <v>85000</v>
       </c>
       <c r="E8" t="n">
-        <v>9000</v>
+        <v>70000</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>3</v>
+          <t>INV-4730-11</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Ready To Bill</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Variance pending customer acceptance.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HSB-FIN-804</t>
+          <t>PRJ-4870</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Treasury support billing</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>69000</v>
+          <t>ERP wave 3 milestone</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
       </c>
       <c r="D9" t="n">
-        <v>41000</v>
+        <v>210000</v>
       </c>
       <c r="E9" t="n">
-        <v>28000</v>
+        <v>60000</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>9</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>INV-4870-18</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Pending Approval</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Large billing hold due to sign-off delay.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSC-CYB-410</t>
+          <t>PRJ-4902</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Security operations billing</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>63000</v>
+          <t>Clinical ingestion baseline</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
       </c>
       <c r="D10" t="n">
-        <v>59000</v>
+        <v>140000</v>
       </c>
       <c r="E10" t="n">
-        <v>4000</v>
+        <v>35000</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
+          <t>INV-4902-04</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Billed</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Billing lag is impacting revenue realization.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSC-NET-870</t>
+          <t>PRJ-5031</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Reliability squad billing</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>61000</v>
+          <t>Security automation release</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
       </c>
       <c r="D11" t="n">
-        <v>54000</v>
+        <v>75000</v>
       </c>
       <c r="E11" t="n">
-        <v>7000</v>
+        <v>75000</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
+          <t>INV-5031-31</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ready To Bill</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Current cycle billing completed.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AZE-ERP-330</t>
+          <t>PRJ-5077</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ERP wave billing</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>59000</v>
+          <t>Reliability squad monthly billing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
       </c>
       <c r="D12" t="n">
-        <v>8000</v>
+        <v>65000</v>
       </c>
       <c r="E12" t="n">
-        <v>51000</v>
+        <v>58000</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>19</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>INV-5077-09</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Minor pending effort remains to be billed.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AZE-DAT-731</t>
+          <t>PRJ-5105</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data ingestion milestone</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>49000</v>
+          <t>Commerce engine go-live</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
       </c>
       <c r="D13" t="n">
-        <v>31000</v>
+        <v>90000</v>
       </c>
       <c r="E13" t="n">
-        <v>18000</v>
+        <v>90000</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
-        <v>5</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>INV-5105-02</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Delayed</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TGT-COM-610</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Commerce release billing</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D14" t="n">
-        <v>62000</v>
-      </c>
-      <c r="E14" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-03-14</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Billed</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TGT-ANA-205</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Analytics sprint billing</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D15" t="n">
-        <v>39000</v>
-      </c>
-      <c r="E15" t="n">
-        <v>11000</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
-        <v>4</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Pending Approval</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Milestone billed on time.</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2404,7 +2450,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Collected Amount</t>
+          <t>Amount Received</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -2424,582 +2470,872 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Overdue Days</t>
+          <t>Client Response Status</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Status Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PEP-AI-101</t>
+          <t>PRJ-4456</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INV-PEP-1042</t>
+          <t>INV-4410</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>90000</v>
+        <v>460000</v>
       </c>
       <c r="D2" t="n">
-        <v>25000</v>
+        <v>460000</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>21</v>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
+          <t>Payment collected within terms.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PEP-DA-204</t>
+          <t>PRJ-4456</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INV-PEP-1079</t>
+          <t>INV-4482</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>78000</v>
+        <v>220000</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>27</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>Client has not responded to the last reminder.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JCI-OPS-310</t>
+          <t>PRJ-4521</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>INV-JCI-2218</t>
+          <t>INV-4521-61</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>62000</v>
+        <v>730000</v>
       </c>
       <c r="D4" t="n">
-        <v>62000</v>
+        <v>640000</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-17</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Promised</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Client committed to clear balance next week.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JCI-CLO-115</t>
+          <t>PRJ-4588</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INV-JCI-2244</t>
+          <t>INV-4588-12</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>55000</v>
+        <v>540000</v>
       </c>
       <c r="D5" t="n">
-        <v>55000</v>
+        <v>410000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Balance is still pending on approved invoice.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>COM-DIG-501</t>
+          <t>PRJ-4620</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INV-COM-3381</t>
+          <t>INV-4620-18</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>68000</v>
+        <v>515000</v>
       </c>
       <c r="D6" t="n">
-        <v>18000</v>
+        <v>360000</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>34</v>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Promised</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>Part-payment received, rest pending approval.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COM-AIO-118</t>
+          <t>PRJ-4711</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INV-COM-3420</t>
+          <t>INV-4711-10</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>54000</v>
+        <v>720000</v>
       </c>
       <c r="D7" t="n">
-        <v>22000</v>
+        <v>720000</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>12</v>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
+          <t>Collected in full.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HSB-DAT-220</t>
+          <t>PRJ-4730</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>INV-HSB-5188</t>
+          <t>INV-4730-08</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>72000</v>
+        <v>535000</v>
       </c>
       <c r="D8" t="n">
-        <v>52000</v>
+        <v>470000</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Promised</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
+          <t>Client confirmed payment processing.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HSB-FIN-804</t>
+          <t>PRJ-4870</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>INV-HSB-5210</t>
+          <t>INV-4870-01</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>69000</v>
+        <v>430000</v>
       </c>
       <c r="D9" t="n">
-        <v>30000</v>
+        <v>180000</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>11</v>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
+          <t>Collections follow-up is ongoing.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSC-CYB-410</t>
+          <t>PRJ-4902</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>INV-CSC-4106</t>
+          <t>INV-4902-07</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>63000</v>
+        <v>325000</v>
       </c>
       <c r="D10" t="n">
-        <v>63000</v>
+        <v>140000</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Collected</t>
+          <t>Client disputes a milestone amount.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSC-NET-870</t>
+          <t>PRJ-5031</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INV-CSC-4138</t>
+          <t>INV-5031-04</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>61000</v>
+        <v>790000</v>
       </c>
       <c r="D11" t="n">
-        <v>48000</v>
+        <v>790000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-03-28</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
+          <t>Collected in full.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AZE-ERP-330</t>
+          <t>PRJ-5077</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>INV-AZE-6124</t>
+          <t>INV-5077-16</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>59000</v>
+        <v>585000</v>
       </c>
       <c r="D12" t="n">
-        <v>15000</v>
+        <v>540000</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-02-22</t>
+          <t>2026-03-21</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>22</v>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Promised</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>Balance expected this cycle.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AZE-DAT-731</t>
+          <t>PRJ-5105</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INV-AZE-6167</t>
+          <t>INV-5105-12</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>49000</v>
+        <v>740000</v>
       </c>
       <c r="D13" t="n">
-        <v>21000</v>
+        <v>740000</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>9</v>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Partially Collected</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TGT-COM-610</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>INV-TGT-7020</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D14" t="n">
-        <v>65000</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2026-03-29</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Collected</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TGT-ANA-205</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>INV-TGT-7051</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026-04-04</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Partially Collected</t>
+          <t>Invoice closed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Agent Key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Metric Key</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Medium Value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>High Value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>revenue_realization</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>forecast_shortfall_ratio</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Revenue shortfall ratio</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Gap between forecast and target used for revenue realization risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>revenue_realization</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>revenue_delay_days</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Revenue update delay</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Days since the last revenue recognition update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>billing_trigger</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>billing_delay_days</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Billing delay</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Days between milestone completion and billing trigger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>billing_trigger</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>unbilled_amount</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pending billable amount</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Unbilled milestone value that should already have triggered invoicing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>unbilled_revenue</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>days_unbilled</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Unbilled aging</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>How long revenue has remained recognized but not billed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>unbilled_revenue</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>unbilled_amount</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Unbilled revenue</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>300000</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Revenue recognized but not yet invoiced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>collection_monitoring</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>overdue_days</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Overdue days</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Days an invoice remains overdue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>collection_monitoring</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>outstanding_balance</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Outstanding balance</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Receivable value still open on the invoice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>revenue_forecasting</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>forecast_gap_ratio</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Forecast gap ratio</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Forecasted shortfall versus target.</t>
         </is>
       </c>
     </row>

</xml_diff>